<commit_message>
se elimina archivo excel
</commit_message>
<xml_diff>
--- a/Profesionales2.xlsx
+++ b/Profesionales2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documentos\Programacion\CentroPediatricoPuertos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A62E61D-A93D-4DE7-A2F5-8DE71B2F4A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80845D6-F0A7-4E30-A962-15EFC3B143A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9EFDC921-82FF-4A69-8FEC-386D123BAB9A}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{9EFDC921-82FF-4A69-8FEC-386D123BAB9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -281,7 +281,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -291,6 +291,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -307,13 +313,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -322,6 +325,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -689,834 +698,835 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="C5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="C6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="C7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="C8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="3" t="s">
+      <c r="C9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" s="3" t="s">
+      <c r="C10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11" s="3" t="s">
+      <c r="C11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="3" t="s">
+      <c r="C12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="3" t="s">
+      <c r="C13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="3" t="s">
+      <c r="C14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="3" t="s">
+      <c r="C15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="3" t="s">
+      <c r="C16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="3" t="s">
+      <c r="C17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="3" t="s">
+      <c r="C18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19" s="3" t="s">
+      <c r="C19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F20" s="3" t="s">
+      <c r="C20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F21" s="3" t="s">
+      <c r="C21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
+      <c r="C22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3" t="s">
+      <c r="C23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F24" s="3"/>
+      <c r="C24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3" t="s">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F25" s="3"/>
+      <c r="C25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3" t="s">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="3" t="s">
+      <c r="C26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3" t="s">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F27" s="3"/>
+      <c r="C27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3" t="s">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F28" s="3"/>
+      <c r="C28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3" t="s">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F29" s="3" t="s">
+      <c r="C29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3" t="s">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F30" s="3" t="s">
+      <c r="C30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3" t="s">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F31" s="3" t="s">
+      <c r="C31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3" t="s">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F32" s="3" t="s">
+      <c r="C32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3" t="s">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F33" s="3" t="s">
+      <c r="C33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3" t="s">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F34" s="3" t="s">
+      <c r="C34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3" t="s">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F35" s="3" t="s">
+      <c r="C35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3" t="s">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F36" s="3" t="s">
+      <c r="C36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3" t="s">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F37" s="3" t="s">
+      <c r="C37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F38" s="3" t="s">
+      <c r="C38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3" t="s">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C39" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F39" s="3" t="s">
+      <c r="C39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3" t="s">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F40" s="3" t="s">
+      <c r="C40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
+      <c r="A41" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F41" s="3" t="s">
+      <c r="C41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C42" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F42" s="3" t="s">
+      <c r="C42" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
+      <c r="A43" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C43" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F43" s="3" t="s">
+      <c r="C43" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3" t="s">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F44" s="3" t="s">
+      <c r="C44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
+      <c r="A45" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C45" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F45" s="3" t="s">
+      <c r="C45" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>